<commit_message>
feat(templates): update EMAX PL template and mapping
根据 /Users/max/Public/.../EMAX PTE-RO PL template.xls 更新：
- .xls → .xlsx 转换（xlrd + openpyxl）
- 新增列：G=Net Weight, I=Gross Weight（原模板只有 Net Weight）
- LineColumns 扩展 net_weight/gross_weight/carton_count/cbm 可选字段
- Renderer 支持按行写入装箱字段
- mapping YAML 配置 style 节（bold: A1, A2; underline: I6）
</commit_message>
<xml_diff>
--- a/templates/emax/pl.xlsx
+++ b/templates/emax/pl.xlsx
@@ -522,10 +522,7 @@
           <t>Invoice No.</t>
         </is>
       </c>
-      <c r="K6">
-        <f>发票号</f>
-        <v/>
-      </c>
+      <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
     </row>
@@ -613,11 +610,7 @@
     <row r="10">
       <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>括号内数值手动更新</t>
-        </is>
-      </c>
+      <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr"/>
@@ -650,50 +643,18 @@
     </row>
     <row r="12">
       <c r="A12" t="inlineStr"/>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>RO new PO template A列"Purchasing Document"</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>RO new PO template J列"Model"</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>RO new PO template I列"Material"</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>PO record</t>
-        </is>
-      </c>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>SK+YM箱单</t>
-        </is>
-      </c>
+      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>SK+YM箱单</t>
-        </is>
-      </c>
+      <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>SK+YM箱单</t>
-        </is>
-      </c>
+      <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>SK+YM箱单</t>
-        </is>
-      </c>
+      <c r="M12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr"/>
@@ -1131,11 +1092,7 @@
         </is>
       </c>
       <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>箱数手动更新</t>
-        </is>
-      </c>
+      <c r="D25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">

</xml_diff>